<commit_message>
Committing after changing the flow to account fo changes in file/log names
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>Rb87/Sr86</t>
   </si>
@@ -64,31 +64,31 @@
     <t>MicaMg-3</t>
   </si>
   <si>
+    <t>MicaMg-4</t>
+  </si>
+  <si>
+    <t>MicaMg-5</t>
+  </si>
+  <si>
     <t>MicaMg-6</t>
   </si>
   <si>
-    <t>MicaMg-4</t>
-  </si>
-  <si>
-    <t>MicaMg-5</t>
-  </si>
-  <si>
     <t>MD4B_V-1</t>
   </si>
   <si>
     <t>MD4B_V-2</t>
   </si>
   <si>
-    <t>MD4B_V-3</t>
-  </si>
-  <si>
-    <t>MD4B_H-1</t>
-  </si>
-  <si>
-    <t>MD4B_H-2</t>
-  </si>
-  <si>
-    <t>MD4B_H-3</t>
+    <t>MD4B_V3</t>
+  </si>
+  <si>
+    <t>MD4B_V4</t>
+  </si>
+  <si>
+    <t>MD4B_V-5</t>
+  </si>
+  <si>
+    <t>MD4B_V-6</t>
   </si>
   <si>
     <t>LaPosta_V-1</t>
@@ -100,31 +100,67 @@
     <t>LaPosta_V-3</t>
   </si>
   <si>
-    <t>LaPosta_H-1</t>
-  </si>
-  <si>
-    <t>LaPosta_H-2</t>
-  </si>
-  <si>
-    <t>LaPosta_H-3</t>
-  </si>
-  <si>
-    <t>Hogsbo_V-1</t>
-  </si>
-  <si>
-    <t>Hogsbo_V-2</t>
-  </si>
-  <si>
-    <t>Hogsbo_V-3</t>
-  </si>
-  <si>
-    <t>Hogsbo_H-1</t>
-  </si>
-  <si>
-    <t>Hogsbo_H-2</t>
-  </si>
-  <si>
-    <t>Hogsbo_H-3</t>
+    <t>LaPosta_V-4</t>
+  </si>
+  <si>
+    <t>LaPosta_V-5</t>
+  </si>
+  <si>
+    <t>MicaFe-1</t>
+  </si>
+  <si>
+    <t>MicaFe-2</t>
+  </si>
+  <si>
+    <t>MicaFe-3</t>
+  </si>
+  <si>
+    <t>MicaFe-4</t>
+  </si>
+  <si>
+    <t>MicaFe-5</t>
+  </si>
+  <si>
+    <t>MicaFe-6</t>
+  </si>
+  <si>
+    <t>HogsboM_V-1</t>
+  </si>
+  <si>
+    <t>HogsboM_V-2</t>
+  </si>
+  <si>
+    <t>HogsboM_V-3</t>
+  </si>
+  <si>
+    <t>HogsboM_V-4</t>
+  </si>
+  <si>
+    <t>HogsboM_V-5</t>
+  </si>
+  <si>
+    <t>BRM1_V-1</t>
+  </si>
+  <si>
+    <t>BRM1_V-2</t>
+  </si>
+  <si>
+    <t>BRM1_V-3</t>
+  </si>
+  <si>
+    <t>BRM2_V-1</t>
+  </si>
+  <si>
+    <t>BRM2_V-2</t>
+  </si>
+  <si>
+    <t>BRM2_V-3</t>
+  </si>
+  <si>
+    <t>BRM2_V-4</t>
+  </si>
+  <si>
+    <t>BRM2_V-5</t>
   </si>
 </sst>
 </file>
@@ -482,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -513,25 +549,25 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>2.494921439301245</v>
+        <v>2.570946498016605</v>
       </c>
       <c r="C2">
-        <v>0.08653397901963951</v>
+        <v>0.06582219137918219</v>
       </c>
       <c r="D2">
-        <v>0.7443934341783814</v>
+        <v>0.5662239000332543</v>
       </c>
       <c r="E2">
-        <v>0.8028336071922046</v>
+        <v>0.7969899999999999</v>
       </c>
       <c r="F2">
-        <v>0.006312865517871274</v>
+        <v>0.004480141391468522</v>
       </c>
       <c r="G2">
-        <v>0.0543053225518262</v>
+        <v>0.03853963349175318</v>
       </c>
       <c r="H2">
-        <v>0.1310940012667118</v>
+        <v>0.1309712264918568</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -539,25 +575,25 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>2.442536004914573</v>
+        <v>2.570946498016617</v>
       </c>
       <c r="C3">
-        <v>0.09810781913967277</v>
+        <v>0.1002268489095608</v>
       </c>
       <c r="D3">
-        <v>0.849638636848458</v>
+        <v>0.8621839548107789</v>
       </c>
       <c r="E3">
-        <v>0.792833749028403</v>
+        <v>0.7969899999999986</v>
       </c>
       <c r="F3">
-        <v>0.006417052538531055</v>
+        <v>0.004336261067476769</v>
       </c>
       <c r="G3">
-        <v>0.05557330515787315</v>
+        <v>0.03730192814524864</v>
       </c>
       <c r="H3">
-        <v>0.2507141378687552</v>
+        <v>-0.2733858348220642</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -565,25 +601,25 @@
         <v>9</v>
       </c>
       <c r="B4">
-        <v>2.592160919385591</v>
+        <v>2.570946498016623</v>
       </c>
       <c r="C4">
-        <v>0.1106290568223613</v>
+        <v>0.0818097243868955</v>
       </c>
       <c r="D4">
-        <v>0.9516671307720935</v>
+        <v>0.7037538591831846</v>
       </c>
       <c r="E4">
-        <v>0.7951868933727421</v>
+        <v>0.7969899999999991</v>
       </c>
       <c r="F4">
-        <v>0.005482362425896812</v>
+        <v>0.003799181604203765</v>
       </c>
       <c r="G4">
-        <v>0.04716106481937726</v>
+        <v>0.03268179590792559</v>
       </c>
       <c r="H4">
-        <v>-0.05878239397302774</v>
+        <v>0.2524513605879022</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -591,25 +627,25 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>2.449403076362916</v>
+        <v>2.570946498016625</v>
       </c>
       <c r="C5">
-        <v>0.1012423546169713</v>
+        <v>0.07676443607109558</v>
       </c>
       <c r="D5">
-        <v>0.8767845103724992</v>
+        <v>0.660352648024664</v>
       </c>
       <c r="E5">
-        <v>0.7990071353113677</v>
+        <v>0.7969899999999988</v>
       </c>
       <c r="F5">
-        <v>0.006754249406735049</v>
+        <v>0.004144831463717191</v>
       </c>
       <c r="G5">
-        <v>0.05849351569728526</v>
+        <v>0.03565518842796767</v>
       </c>
       <c r="H5">
-        <v>0.1872471028454815</v>
+        <v>0.03520549354796747</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -617,25 +653,25 @@
         <v>11</v>
       </c>
       <c r="B6">
-        <v>2.508676492371395</v>
+        <v>2.570946498016691</v>
       </c>
       <c r="C6">
-        <v>0.09480782082818742</v>
+        <v>0.04945596989187016</v>
       </c>
       <c r="D6">
-        <v>0.8155677126235669</v>
+        <v>0.425436339406934</v>
       </c>
       <c r="E6">
-        <v>0.7913565661493167</v>
+        <v>0.7969899999999978</v>
       </c>
       <c r="F6">
-        <v>0.006986024364486179</v>
+        <v>0.003565295218268958</v>
       </c>
       <c r="G6">
-        <v>0.06009605390679486</v>
+        <v>0.03066982914058131</v>
       </c>
       <c r="H6">
-        <v>0.2717204060587994</v>
+        <v>-0.03197547177535697</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -643,25 +679,25 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>2.447230409301052</v>
+        <v>2.570946498016675</v>
       </c>
       <c r="C7">
-        <v>0.0869093595848032</v>
+        <v>0.07950935705303436</v>
       </c>
       <c r="D7">
-        <v>0.7476225798988458</v>
+        <v>0.6839653511436313</v>
       </c>
       <c r="E7">
-        <v>0.8007220489459657</v>
+        <v>0.7969899999999983</v>
       </c>
       <c r="F7">
-        <v>0.006586876297099498</v>
+        <v>0.004661903771521268</v>
       </c>
       <c r="G7">
-        <v>0.05666245240142319</v>
+        <v>0.04010321260627872</v>
       </c>
       <c r="H7">
-        <v>0.02026821406463038</v>
+        <v>-0.07939173129678218</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -669,25 +705,25 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>186.1245103346817</v>
+        <v>178.3461106185524</v>
       </c>
       <c r="C8">
-        <v>8.43408451526151</v>
+        <v>6.500853284864617</v>
       </c>
       <c r="D8">
-        <v>73.04131447881431</v>
+        <v>55.92245446972795</v>
       </c>
       <c r="E8">
-        <v>2.056226722243069</v>
+        <v>2.053228123679203</v>
       </c>
       <c r="F8">
-        <v>0.03549980309674478</v>
+        <v>0.02335533559556806</v>
       </c>
       <c r="G8">
-        <v>0.3074373131112646</v>
+        <v>0.2009101935140152</v>
       </c>
       <c r="H8">
-        <v>-0.3960008822069707</v>
+        <v>0.3048969575552816</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -695,25 +731,25 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>180.7442346502985</v>
+        <v>193.670421218785</v>
       </c>
       <c r="C9">
-        <v>7.262673946877269</v>
+        <v>4.119885700125201</v>
       </c>
       <c r="D9">
-        <v>62.8966013739911</v>
+        <v>35.44059685551461</v>
       </c>
       <c r="E9">
-        <v>2.088407639534927</v>
+        <v>2.070360763580756</v>
       </c>
       <c r="F9">
-        <v>0.0943454207074281</v>
+        <v>0.01919274916959427</v>
       </c>
       <c r="G9">
-        <v>0.8170553106336317</v>
+        <v>0.1651022711256122</v>
       </c>
       <c r="H9">
-        <v>-0.6445087433114871</v>
+        <v>0.309631706988087</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -721,25 +757,25 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>182.7558526390436</v>
+        <v>183.3766817213902</v>
       </c>
       <c r="C10">
-        <v>7.308268151460369</v>
+        <v>3.967847534144779</v>
       </c>
       <c r="D10">
-        <v>63.29145876833419</v>
+        <v>34.13271509874642</v>
       </c>
       <c r="E10">
-        <v>2.073407387920274</v>
+        <v>2.063065303235316</v>
       </c>
       <c r="F10">
-        <v>0.0283071818172551</v>
+        <v>0.01864072263393244</v>
       </c>
       <c r="G10">
-        <v>0.2451473856328787</v>
+        <v>0.1603535593098104</v>
       </c>
       <c r="H10">
-        <v>-0.4291087281633629</v>
+        <v>0.1811722986500531</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -747,25 +783,25 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>192.5911418698248</v>
+        <v>181.151133508252</v>
       </c>
       <c r="C11">
-        <v>7.587052370755097</v>
+        <v>4.300629895596128</v>
       </c>
       <c r="D11">
-        <v>65.70580092916866</v>
+        <v>36.99541721508546</v>
       </c>
       <c r="E11">
-        <v>2.075303296813821</v>
+        <v>2.072837843933319</v>
       </c>
       <c r="F11">
-        <v>0.02523633642893184</v>
+        <v>0.01718912911571038</v>
       </c>
       <c r="G11">
-        <v>0.2185530844590564</v>
+        <v>0.1478664797105335</v>
       </c>
       <c r="H11">
-        <v>-0.04345566632044449</v>
+        <v>0.1589255060021761</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -773,25 +809,25 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>183.7533705048996</v>
+        <v>187.050696726685</v>
       </c>
       <c r="C12">
-        <v>6.856851126340165</v>
+        <v>4.363802519941109</v>
       </c>
       <c r="D12">
-        <v>59.38207265378525</v>
+        <v>37.53884867767368</v>
       </c>
       <c r="E12">
-        <v>2.076247457520819</v>
+        <v>2.060824505107423</v>
       </c>
       <c r="F12">
-        <v>0.02786742336102768</v>
+        <v>0.0178311674534386</v>
       </c>
       <c r="G12">
-        <v>0.2413389656866589</v>
+        <v>0.153389502325583</v>
       </c>
       <c r="H12">
-        <v>-0.227408482858362</v>
+        <v>0.1567534860850645</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -799,25 +835,25 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>182.5190752576984</v>
+        <v>182.8336705407285</v>
       </c>
       <c r="C13">
-        <v>6.880497376672017</v>
+        <v>4.708207157316349</v>
       </c>
       <c r="D13">
-        <v>59.58685518870155</v>
+        <v>40.50152939185337</v>
       </c>
       <c r="E13">
-        <v>2.060449150977407</v>
+        <v>2.094725055703427</v>
       </c>
       <c r="F13">
-        <v>0.02881745394273413</v>
+        <v>0.01806365881715744</v>
       </c>
       <c r="G13">
-        <v>0.2495664718679579</v>
+        <v>0.1553894686580707</v>
       </c>
       <c r="H13">
-        <v>-0.5266900456218511</v>
+        <v>0.2699415941829031</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -825,25 +861,25 @@
         <v>19</v>
       </c>
       <c r="B14">
-        <v>97.36707714999383</v>
+        <v>96.57843274196253</v>
       </c>
       <c r="C14">
-        <v>2.666871209879327</v>
+        <v>1.658122423167146</v>
       </c>
       <c r="D14">
-        <v>23.09578216376839</v>
+        <v>14.26370841666069</v>
       </c>
       <c r="E14">
-        <v>0.9129531641452021</v>
+        <v>0.9165895194814084</v>
       </c>
       <c r="F14">
-        <v>0.01644875712575511</v>
+        <v>0.0108918014900254</v>
       </c>
       <c r="G14">
-        <v>0.1424504153158423</v>
+        <v>0.09369481916125799</v>
       </c>
       <c r="H14">
-        <v>0.01260925900322776</v>
+        <v>0.2219273082623935</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -851,25 +887,25 @@
         <v>20</v>
       </c>
       <c r="B15">
-        <v>91.28786239174904</v>
+        <v>107.56798881755</v>
       </c>
       <c r="C15">
-        <v>2.571101256639932</v>
+        <v>1.922577960870714</v>
       </c>
       <c r="D15">
-        <v>22.26639003952275</v>
+        <v>16.53864097065743</v>
       </c>
       <c r="E15">
-        <v>0.9166908167495607</v>
+        <v>0.9180649697075086</v>
       </c>
       <c r="F15">
-        <v>0.01372552370240204</v>
+        <v>0.01303145295899664</v>
       </c>
       <c r="G15">
-        <v>0.1188665220652561</v>
+        <v>0.1121007970554542</v>
       </c>
       <c r="H15">
-        <v>0.06711837804976839</v>
+        <v>0.02419026911873125</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -877,25 +913,25 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>81.21406212937526</v>
+        <v>58.75479339134198</v>
       </c>
       <c r="C16">
-        <v>2.255355164235859</v>
+        <v>1.064064336970629</v>
       </c>
       <c r="D16">
-        <v>19.53194866784679</v>
+        <v>9.153427531681402</v>
       </c>
       <c r="E16">
-        <v>0.8958137945515493</v>
+        <v>0.8796716076311411</v>
       </c>
       <c r="F16">
-        <v>0.01180223865493408</v>
+        <v>0.008065869537556525</v>
       </c>
       <c r="G16">
-        <v>0.102210384966996</v>
+        <v>0.06938523332359192</v>
       </c>
       <c r="H16">
-        <v>0.09852983610829349</v>
+        <v>0.2510764540123643</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -903,25 +939,25 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>88.30857896729363</v>
+        <v>58.92134626130558</v>
       </c>
       <c r="C17">
-        <v>3.446122242343916</v>
+        <v>1.012045437106633</v>
       </c>
       <c r="D17">
-        <v>29.84429406416426</v>
+        <v>8.705944035017584</v>
       </c>
       <c r="E17">
-        <v>0.9133036404750527</v>
+        <v>0.8784406053849807</v>
       </c>
       <c r="F17">
-        <v>0.01750802858677359</v>
+        <v>0.008936309211949517</v>
       </c>
       <c r="G17">
-        <v>0.151623975263301</v>
+        <v>0.07687303852805911</v>
       </c>
       <c r="H17">
-        <v>0.1508897772189429</v>
+        <v>0.02430846820693065</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -929,25 +965,25 @@
         <v>23</v>
       </c>
       <c r="B18">
-        <v>90.65973720514188</v>
+        <v>43.26347477017217</v>
       </c>
       <c r="C18">
-        <v>2.930635595056279</v>
+        <v>0.8184954959685709</v>
       </c>
       <c r="D18">
-        <v>25.38004874553663</v>
+        <v>7.040964485931023</v>
       </c>
       <c r="E18">
-        <v>0.8972352168779207</v>
+        <v>0.9020695880391795</v>
       </c>
       <c r="F18">
-        <v>0.01262241397861893</v>
+        <v>0.007706903803393745</v>
       </c>
       <c r="G18">
-        <v>0.109313311625678</v>
+        <v>0.06629729331860093</v>
       </c>
       <c r="H18">
-        <v>0.1657102456271982</v>
+        <v>0.1302947897386202</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -955,25 +991,25 @@
         <v>24</v>
       </c>
       <c r="B19">
-        <v>78.60583790628458</v>
+        <v>39.42486012330251</v>
       </c>
       <c r="C19">
-        <v>2.209941351783893</v>
+        <v>0.8665151685881772</v>
       </c>
       <c r="D19">
-        <v>19.13865351518574</v>
+        <v>7.454045329021779</v>
       </c>
       <c r="E19">
-        <v>0.9100702288352225</v>
+        <v>0.9132983545928197</v>
       </c>
       <c r="F19">
-        <v>0.03509141039562877</v>
+        <v>0.009631787693890406</v>
       </c>
       <c r="G19">
-        <v>0.3039005285723986</v>
+        <v>0.08285577064594367</v>
       </c>
       <c r="H19">
-        <v>-0.1360258561310173</v>
+        <v>0.1862477042440946</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -981,25 +1017,25 @@
         <v>25</v>
       </c>
       <c r="B20">
-        <v>879.1726939227149</v>
+        <v>853.3600526912761</v>
       </c>
       <c r="C20">
-        <v>27.5024365984987</v>
+        <v>101.1508308704687</v>
       </c>
       <c r="D20">
-        <v>238.1780876027076</v>
+        <v>870.1323481793885</v>
       </c>
       <c r="E20">
-        <v>2.009354736824872</v>
+        <v>1.766442941258061</v>
       </c>
       <c r="F20">
-        <v>0.08179388408802907</v>
+        <v>0.14648023025448</v>
       </c>
       <c r="G20">
-        <v>0.7083558149443295</v>
+        <v>1.260070585840335</v>
       </c>
       <c r="H20">
-        <v>0.5570929040457984</v>
+        <v>0.904733250520167</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1007,25 +1043,25 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>859.427893914877</v>
+        <v>1413.447089450593</v>
       </c>
       <c r="C21">
-        <v>25.38302685645951</v>
+        <v>58.30775176876982</v>
       </c>
       <c r="D21">
-        <v>219.823460826366</v>
+        <v>501.582246304938</v>
       </c>
       <c r="E21">
-        <v>1.925596145769521</v>
+        <v>2.263790403288942</v>
       </c>
       <c r="F21">
-        <v>0.08257196887402306</v>
+        <v>0.07076901804891719</v>
       </c>
       <c r="G21">
-        <v>0.7150942268540192</v>
+        <v>0.6087781120859961</v>
       </c>
       <c r="H21">
-        <v>0.5647603795052714</v>
+        <v>0.4257684772558101</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1033,25 +1069,25 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>935.5421275005007</v>
+        <v>294.3950723310982</v>
       </c>
       <c r="C22">
-        <v>25.92001639974653</v>
+        <v>10.59758670881693</v>
       </c>
       <c r="D22">
-        <v>224.4739266868976</v>
+        <v>91.16388791493098</v>
       </c>
       <c r="E22">
-        <v>2.087052856589373</v>
+        <v>1.123289271828217</v>
       </c>
       <c r="F22">
-        <v>0.08034925748521622</v>
+        <v>0.02292278935103359</v>
       </c>
       <c r="G22">
-        <v>0.6958449815741421</v>
+        <v>0.1971892900254919</v>
       </c>
       <c r="H22">
-        <v>0.6232933724874744</v>
+        <v>-0.044400725338273</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1059,25 +1095,25 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>869.9308080685487</v>
+        <v>289.1545093411332</v>
       </c>
       <c r="C23">
-        <v>56.07909863569802</v>
+        <v>10.39440228681137</v>
       </c>
       <c r="D23">
-        <v>485.6592403984775</v>
+        <v>89.41602942764308</v>
       </c>
       <c r="E23">
-        <v>1.857148591634332</v>
+        <v>1.123299801315643</v>
       </c>
       <c r="F23">
-        <v>0.1505270848392299</v>
+        <v>0.02258797875192223</v>
       </c>
       <c r="G23">
-        <v>1.303602794283885</v>
+        <v>0.1943091403490826</v>
       </c>
       <c r="H23">
-        <v>-0.130446015061649</v>
+        <v>0.1422967310430169</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1085,25 +1121,25 @@
         <v>29</v>
       </c>
       <c r="B24">
-        <v>907.2557956853623</v>
+        <v>1271.179491288408</v>
       </c>
       <c r="C24">
-        <v>45.16061083088314</v>
+        <v>42.55565745862245</v>
       </c>
       <c r="D24">
-        <v>388.4862636255849</v>
+        <v>366.0776074119189</v>
       </c>
       <c r="E24">
-        <v>1.869166657263008</v>
+        <v>2.346539061462481</v>
       </c>
       <c r="F24">
-        <v>0.07953497762673628</v>
+        <v>0.08384015799047768</v>
       </c>
       <c r="G24">
-        <v>0.6841857476521435</v>
+        <v>0.7212203094743319</v>
       </c>
       <c r="H24">
-        <v>-0.1064935314123294</v>
+        <v>0.4824042790124707</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1111,25 +1147,25 @@
         <v>30</v>
       </c>
       <c r="B25">
-        <v>18.80849713397902</v>
+        <v>2184.670863820465</v>
       </c>
       <c r="C25">
-        <v>13.14910950937785</v>
+        <v>83.36421917418376</v>
       </c>
       <c r="D25">
-        <v>60.25678964798762</v>
+        <v>717.1261289693604</v>
       </c>
       <c r="E25">
-        <v>0.7986312899465969</v>
+        <v>9.300031713507376</v>
       </c>
       <c r="F25">
-        <v>0.03269649863881074</v>
+        <v>0.2477773588882345</v>
       </c>
       <c r="G25">
-        <v>0.1498341799723708</v>
+        <v>2.131461434965348</v>
       </c>
       <c r="H25">
-        <v>0.9490677797231796</v>
+        <v>0.6968762274792842</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1137,25 +1173,25 @@
         <v>31</v>
       </c>
       <c r="B26">
-        <v>26252.74740516192</v>
+        <v>2176.031937231136</v>
       </c>
       <c r="C26">
-        <v>1843.766685076248</v>
+        <v>78.90721913865009</v>
       </c>
       <c r="D26">
-        <v>15967.48787927454</v>
+        <v>678.7855649484792</v>
       </c>
       <c r="E26">
-        <v>383.3045655046755</v>
+        <v>9.09918555034626</v>
       </c>
       <c r="F26">
-        <v>27.28473716383073</v>
+        <v>0.2422940005167107</v>
       </c>
       <c r="G26">
-        <v>236.2927551945879</v>
+        <v>2.08429180269774</v>
       </c>
       <c r="H26">
-        <v>0.9270083311616732</v>
+        <v>0.6839860192277387</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1163,25 +1199,25 @@
         <v>32</v>
       </c>
       <c r="B27">
-        <v>22751.16035240731</v>
+        <v>2034.01561238801</v>
       </c>
       <c r="C27">
-        <v>1329.911137443451</v>
+        <v>71.10187846825968</v>
       </c>
       <c r="D27">
-        <v>11517.36829801886</v>
+        <v>611.6414856817044</v>
       </c>
       <c r="E27">
-        <v>325.5281218533489</v>
+        <v>9.713119184727631</v>
       </c>
       <c r="F27">
-        <v>14.40432909030317</v>
+        <v>0.2614113208950758</v>
       </c>
       <c r="G27">
-        <v>124.7451491667374</v>
+        <v>2.248745210826699</v>
       </c>
       <c r="H27">
-        <v>0.7522523682969079</v>
+        <v>0.8426014574283645</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1189,25 +1225,25 @@
         <v>33</v>
       </c>
       <c r="B28">
-        <v>25999.78835589021</v>
+        <v>1942.799865121578</v>
       </c>
       <c r="C28">
-        <v>1687.943298296558</v>
+        <v>52.78384554143345</v>
       </c>
       <c r="D28">
-        <v>14618.01776472514</v>
+        <v>454.0638081927482</v>
       </c>
       <c r="E28">
-        <v>374.5326728927204</v>
+        <v>9.410152988001752</v>
       </c>
       <c r="F28">
-        <v>23.20723078773742</v>
+        <v>0.1663732075733748</v>
       </c>
       <c r="G28">
-        <v>200.9805141366896</v>
+        <v>1.43119644726737</v>
       </c>
       <c r="H28">
-        <v>0.8255248626201845</v>
+        <v>0.5713704898243415</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1215,25 +1251,25 @@
         <v>34</v>
       </c>
       <c r="B29">
-        <v>16737.61387961584</v>
+        <v>1939.957893840889</v>
       </c>
       <c r="C29">
-        <v>10018.85812064888</v>
+        <v>60.14431316620439</v>
       </c>
       <c r="D29">
-        <v>86765.85649393953</v>
+        <v>517.3809448185646</v>
       </c>
       <c r="E29">
-        <v>314.0219121293765</v>
+        <v>9.833236150997914</v>
       </c>
       <c r="F29">
-        <v>35.29778449646336</v>
+        <v>0.2388649185695426</v>
       </c>
       <c r="G29">
-        <v>305.6877807124578</v>
+        <v>2.054793724420855</v>
       </c>
       <c r="H29">
-        <v>0.426339969307021</v>
+        <v>0.6578213157765926</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1241,22 +1277,25 @@
         <v>35</v>
       </c>
       <c r="B30">
-        <v>-16336.64476158242</v>
+        <v>1606.65666867318</v>
       </c>
       <c r="C30">
-        <v>105387.785341679</v>
+        <v>46.27384535268702</v>
       </c>
       <c r="D30">
-        <v>906580.0086823896</v>
+        <v>398.0626690806426</v>
       </c>
       <c r="E30">
-        <v>391.9796005964352</v>
+        <v>9.355771055438691</v>
       </c>
       <c r="F30">
-        <v>21.58256378494409</v>
+        <v>0.2142233133405674</v>
       </c>
       <c r="G30">
-        <v>185.6602337747837</v>
+        <v>1.842818621139153</v>
+      </c>
+      <c r="H30">
+        <v>0.7761351914952238</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1264,25 +1303,337 @@
         <v>36</v>
       </c>
       <c r="B31">
-        <v>11732.34119111122</v>
+        <v>16155.81471500207</v>
       </c>
       <c r="C31">
-        <v>15681.48700530968</v>
+        <v>1521.492565905861</v>
       </c>
       <c r="D31">
-        <v>135805.6611571375</v>
+        <v>13088.37394330951</v>
       </c>
       <c r="E31">
-        <v>301.9140221408573</v>
+        <v>200.8564070748143</v>
       </c>
       <c r="F31">
-        <v>33.16826871161712</v>
+        <v>19.34656980542374</v>
       </c>
       <c r="G31">
-        <v>287.2456330380898</v>
+        <v>166.4254862678006</v>
       </c>
       <c r="H31">
-        <v>0.3097467839510151</v>
+        <v>0.7221076767644226</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32">
+        <v>18307.02324260013</v>
+      </c>
+      <c r="C32">
+        <v>928.2212914716906</v>
+      </c>
+      <c r="D32">
+        <v>7984.861469033863</v>
+      </c>
+      <c r="E32">
+        <v>217.1934913658665</v>
+      </c>
+      <c r="F32">
+        <v>18.9267487185441</v>
+      </c>
+      <c r="G32">
+        <v>162.8140487244986</v>
+      </c>
+      <c r="H32">
+        <v>0.1538184555886099</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33">
+        <v>19006.4995079856</v>
+      </c>
+      <c r="C33">
+        <v>865.7590106912226</v>
+      </c>
+      <c r="D33">
+        <v>7447.540612838931</v>
+      </c>
+      <c r="E33">
+        <v>229.1648891391098</v>
+      </c>
+      <c r="F33">
+        <v>23.01132671457044</v>
+      </c>
+      <c r="G33">
+        <v>197.9509172249223</v>
+      </c>
+      <c r="H33">
+        <v>0.4401350705722868</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34">
+        <v>17140.05214666761</v>
+      </c>
+      <c r="C34">
+        <v>898.616612220899</v>
+      </c>
+      <c r="D34">
+        <v>7730.192388692086</v>
+      </c>
+      <c r="E34">
+        <v>211.3014988611413</v>
+      </c>
+      <c r="F34">
+        <v>22.17865107766293</v>
+      </c>
+      <c r="G34">
+        <v>190.787970554302</v>
+      </c>
+      <c r="H34">
+        <v>0.4867787669387967</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35">
+        <v>12687.89849881931</v>
+      </c>
+      <c r="C35">
+        <v>665.0800385141349</v>
+      </c>
+      <c r="D35">
+        <v>5682.446340000696</v>
+      </c>
+      <c r="E35">
+        <v>159.3439158823562</v>
+      </c>
+      <c r="F35">
+        <v>13.94921749685544</v>
+      </c>
+      <c r="G35">
+        <v>119.1821665373817</v>
+      </c>
+      <c r="H35">
+        <v>0.5385797232910583</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36">
+        <v>250.4189459803449</v>
+      </c>
+      <c r="C36">
+        <v>6.125539335265054</v>
+      </c>
+      <c r="D36">
+        <v>52.69388179801407</v>
+      </c>
+      <c r="E36">
+        <v>2.411190016309578</v>
+      </c>
+      <c r="F36">
+        <v>0.08947606138806991</v>
+      </c>
+      <c r="G36">
+        <v>0.7697021836740509</v>
+      </c>
+      <c r="H36">
+        <v>0.4861414862115565</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37">
+        <v>245.2540951429783</v>
+      </c>
+      <c r="C37">
+        <v>13.81017782992817</v>
+      </c>
+      <c r="D37">
+        <v>118.799641688743</v>
+      </c>
+      <c r="E37">
+        <v>2.380598945909948</v>
+      </c>
+      <c r="F37">
+        <v>0.08053429977627624</v>
+      </c>
+      <c r="G37">
+        <v>0.6927822418290465</v>
+      </c>
+      <c r="H37">
+        <v>-0.1134836087156965</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38">
+        <v>263.1238808954787</v>
+      </c>
+      <c r="C38">
+        <v>8.470618124263396</v>
+      </c>
+      <c r="D38">
+        <v>72.86701231782023</v>
+      </c>
+      <c r="E38">
+        <v>2.453409915234906</v>
+      </c>
+      <c r="F38">
+        <v>0.08365632005971013</v>
+      </c>
+      <c r="G38">
+        <v>0.7196388757974495</v>
+      </c>
+      <c r="H38">
+        <v>0.4778240242488693</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39">
+        <v>285.0327326037122</v>
+      </c>
+      <c r="C39">
+        <v>6.387107578363</v>
+      </c>
+      <c r="D39">
+        <v>54.94397690467147</v>
+      </c>
+      <c r="E39">
+        <v>2.943100347582496</v>
+      </c>
+      <c r="F39">
+        <v>0.1016924894402733</v>
+      </c>
+      <c r="G39">
+        <v>0.8747918713805285</v>
+      </c>
+      <c r="H39">
+        <v>0.4144883888084265</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40">
+        <v>288.352201749955</v>
+      </c>
+      <c r="C40">
+        <v>6.905205979335607</v>
+      </c>
+      <c r="D40">
+        <v>59.40082787017251</v>
+      </c>
+      <c r="E40">
+        <v>2.943233227005778</v>
+      </c>
+      <c r="F40">
+        <v>0.09668693686881222</v>
+      </c>
+      <c r="G40">
+        <v>0.8317324800195387</v>
+      </c>
+      <c r="H40">
+        <v>0.5442267952081947</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41">
+        <v>302.7998450392808</v>
+      </c>
+      <c r="C41">
+        <v>8.060498396452946</v>
+      </c>
+      <c r="D41">
+        <v>69.33902902076375</v>
+      </c>
+      <c r="E41">
+        <v>3.061488669386628</v>
+      </c>
+      <c r="F41">
+        <v>0.1080425464684174</v>
+      </c>
+      <c r="G41">
+        <v>0.9294171274008943</v>
+      </c>
+      <c r="H41">
+        <v>0.6844615397848718</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42">
+        <v>306.3235046465668</v>
+      </c>
+      <c r="C42">
+        <v>8.303586080740523</v>
+      </c>
+      <c r="D42">
+        <v>71.43014834941766</v>
+      </c>
+      <c r="E42">
+        <v>3.032934523935971</v>
+      </c>
+      <c r="F42">
+        <v>0.1012570782041991</v>
+      </c>
+      <c r="G42">
+        <v>0.8710463223028931</v>
+      </c>
+      <c r="H42">
+        <v>0.03739607752232441</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43">
+        <v>304.7192277517945</v>
+      </c>
+      <c r="C43">
+        <v>5.99449031544735</v>
+      </c>
+      <c r="D43">
+        <v>51.56655550361506</v>
+      </c>
+      <c r="E43">
+        <v>3.076898438003519</v>
+      </c>
+      <c r="F43">
+        <v>0.1047797096994507</v>
+      </c>
+      <c r="G43">
+        <v>0.9013491442209765</v>
+      </c>
+      <c r="H43">
+        <v>0.2203668102585778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>